<commit_message>
J1 in BOM updated
</commit_message>
<xml_diff>
--- a/Design-Files/Control-Board-v4.0/BOM/Client-BOM-Control-Board-v4.0.xlsx
+++ b/Design-Files/Control-Board-v4.0/BOM/Client-BOM-Control-Board-v4.0.xlsx
@@ -1,20 +1,35 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
-  <workbookPr codeName="ThisWorkbook" defaultThemeVersion="153222"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="24334"/>
+  <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Iftikhar Ahmed\OneDrive\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\eSpark-Consultants\ChristianRaun-EthercatDesign\Design-Files\Control-Board-v4.0\BOM\"/>
     </mc:Choice>
   </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1AB7649F-5294-484B-9C07-4EA030126116}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="24240" windowHeight="13140" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="162913"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
+      <xlwcv:version setVersion="1"/>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
@@ -186,9 +201,6 @@
     <t>15A@8/20us 9V 5V 3.3V Unidirectional SOD-323 TVS ROHS</t>
   </si>
   <si>
-    <t>Gold 250V 1A Right-Angle Square Pins 1mm 10P 260℃ 4mm -40℃~+105℃ 1.27mm 双排 Black Brass 1.27mm 2x5P Push-Pull,P=1.27mm Pin Headers ROHS</t>
-  </si>
-  <si>
     <t>CONN RCPT 1.27MM SMD 32POS</t>
   </si>
   <si>
@@ -276,9 +288,6 @@
     <t>SOD-323</t>
   </si>
   <si>
-    <t>X1321WR-2x05J-C40D18</t>
-  </si>
-  <si>
     <t>M55-6013242R</t>
   </si>
   <si>
@@ -517,12 +526,18 @@
   </si>
   <si>
     <t>IC</t>
+  </si>
+  <si>
+    <t>X6521WR-2x05H-C60D30</t>
+  </si>
+  <si>
+    <t>Gold 250V 3A Pin Header 2.5mm 10P -40℃~+105℃ 2.54mm 2 Black Brass 2x5P 2.54mm Through Hole,Right Angle,P=2.54mm Pin Headers ROHS</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="8" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -736,9 +751,6 @@
     <xf numFmtId="0" fontId="5" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="6" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -750,6 +762,9 @@
     </xf>
     <xf numFmtId="0" fontId="6" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1036,24 +1051,24 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr codeName="Sheet1"/>
   <dimension ref="A1:K34"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="3.140625" style="4" customWidth="1"/>
-    <col min="3" max="3" width="18.7109375" style="4" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="3.109375" style="4" customWidth="1"/>
+    <col min="3" max="3" width="18.6640625" style="4" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="36" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="30" customWidth="1"/>
-    <col min="6" max="6" width="26.5703125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="33.42578125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="21.42578125" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="17.85546875" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="16.7109375" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="29.42578125" customWidth="1"/>
+    <col min="6" max="6" width="26.5546875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="33.44140625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="21.44140625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="17.88671875" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="16.6640625" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="29.44140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A1" s="1"/>
       <c r="B1" s="3"/>
       <c r="C1" s="3"/>
@@ -1062,11 +1077,11 @@
       <c r="F1" s="2"/>
       <c r="G1" s="2"/>
       <c r="H1" s="2"/>
-      <c r="I1" s="14"/>
-      <c r="J1" s="14"/>
-      <c r="K1" s="14"/>
-    </row>
-    <row r="2" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="I1" s="18"/>
+      <c r="J1" s="18"/>
+      <c r="K1" s="18"/>
+    </row>
+    <row r="2" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A2" s="1"/>
       <c r="B2" s="5" t="s">
         <v>0</v>
@@ -1081,25 +1096,25 @@
         <v>45</v>
       </c>
       <c r="F2" s="5" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="G2" s="6" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="H2" s="5" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="I2" s="6" t="s">
-        <v>163</v>
+        <v>161</v>
       </c>
       <c r="J2" s="5" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="K2" s="5" t="s">
-        <v>164</v>
-      </c>
-    </row>
-    <row r="3" spans="1:11" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11" ht="24.6" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A3" s="1"/>
       <c r="B3" s="11">
         <f>ROW(B3) - ROW($B$2)</f>
@@ -1115,23 +1130,23 @@
         <v>46</v>
       </c>
       <c r="F3" s="7" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="G3" s="8" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="H3" s="7" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
       <c r="I3" s="8" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="J3" s="7">
         <v>21</v>
       </c>
       <c r="K3" s="7"/>
     </row>
-    <row r="4" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A4" s="1"/>
       <c r="B4" s="11">
         <f t="shared" ref="B4:B34" si="0">ROW(B4) - ROW($B$2)</f>
@@ -1147,23 +1162,23 @@
         <v>47</v>
       </c>
       <c r="F4" s="9" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="G4" s="10" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="H4" s="9" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="I4" s="10" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="J4" s="9">
         <v>4</v>
       </c>
       <c r="K4" s="9"/>
     </row>
-    <row r="5" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A5" s="1"/>
       <c r="B5" s="11">
         <f>ROW(B5) - ROW($B$2)</f>
@@ -1179,23 +1194,23 @@
         <v>48</v>
       </c>
       <c r="F5" s="7" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="G5" s="8" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="H5" s="7" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
       <c r="I5" s="8" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
       <c r="J5" s="7">
         <v>4</v>
       </c>
       <c r="K5" s="7"/>
     </row>
-    <row r="6" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A6" s="1"/>
       <c r="B6" s="11">
         <f t="shared" si="0"/>
@@ -1211,23 +1226,23 @@
         <v>49</v>
       </c>
       <c r="F6" s="9" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="G6" s="10" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="H6" s="9" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
       <c r="I6" s="10" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="J6" s="9">
         <v>4</v>
       </c>
       <c r="K6" s="9"/>
     </row>
-    <row r="7" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A7" s="1"/>
       <c r="B7" s="11">
         <f>ROW(B7) - ROW($B$2)</f>
@@ -1243,23 +1258,23 @@
         <v>50</v>
       </c>
       <c r="F7" s="7" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="G7" s="8" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="H7" s="7" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="I7" s="8" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="J7" s="7">
         <v>1</v>
       </c>
       <c r="K7" s="7"/>
     </row>
-    <row r="8" spans="1:11" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A8" s="1"/>
       <c r="B8" s="11">
         <f t="shared" si="0"/>
@@ -1275,23 +1290,23 @@
         <v>51</v>
       </c>
       <c r="F8" s="9" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="G8" s="10" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="H8" s="9" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="I8" s="10" t="s">
-        <v>159</v>
+        <v>157</v>
       </c>
       <c r="J8" s="9">
         <v>2</v>
       </c>
       <c r="K8" s="9"/>
     </row>
-    <row r="9" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A9" s="1"/>
       <c r="B9" s="11">
         <f>ROW(B9) - ROW($B$2)</f>
@@ -1307,23 +1322,23 @@
         <v>52</v>
       </c>
       <c r="F9" s="7" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="G9" s="8" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="H9" s="7" t="s">
+        <v>155</v>
+      </c>
+      <c r="I9" s="10" t="s">
         <v>157</v>
-      </c>
-      <c r="I9" s="10" t="s">
-        <v>159</v>
       </c>
       <c r="J9" s="7">
         <v>1</v>
       </c>
       <c r="K9" s="7"/>
     </row>
-    <row r="10" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A10" s="1"/>
       <c r="B10" s="11">
         <f t="shared" si="0"/>
@@ -1339,23 +1354,23 @@
         <v>53</v>
       </c>
       <c r="F10" s="9" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="G10" s="10" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="H10" s="7" t="s">
+        <v>155</v>
+      </c>
+      <c r="I10" s="10" t="s">
         <v>157</v>
-      </c>
-      <c r="I10" s="10" t="s">
-        <v>159</v>
       </c>
       <c r="J10" s="9">
         <v>1</v>
       </c>
       <c r="K10" s="9"/>
     </row>
-    <row r="11" spans="1:11" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:11" ht="24.6" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A11" s="1"/>
       <c r="B11" s="11">
         <f>ROW(B11) - ROW($B$2)</f>
@@ -1371,23 +1386,23 @@
         <v>54</v>
       </c>
       <c r="F11" s="7" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="G11" s="8" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="H11" s="7" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="I11" s="10" t="s">
-        <v>159</v>
+        <v>157</v>
       </c>
       <c r="J11" s="7">
         <v>1</v>
       </c>
       <c r="K11" s="7"/>
     </row>
-    <row r="12" spans="1:11" ht="60.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:11" ht="48.6" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A12" s="1"/>
       <c r="B12" s="11">
         <f t="shared" si="0"/>
@@ -1400,26 +1415,26 @@
         <v>22</v>
       </c>
       <c r="E12" s="10" t="s">
-        <v>55</v>
+        <v>165</v>
       </c>
       <c r="F12" s="9" t="s">
-        <v>158</v>
+        <v>156</v>
       </c>
       <c r="G12" s="10" t="s">
-        <v>85</v>
+        <v>164</v>
       </c>
       <c r="H12" s="9" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="I12" s="10" t="s">
-        <v>159</v>
+        <v>157</v>
       </c>
       <c r="J12" s="9">
         <v>1</v>
       </c>
       <c r="K12" s="9"/>
     </row>
-    <row r="13" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A13" s="1"/>
       <c r="B13" s="11">
         <f>ROW(B13) - ROW($B$2)</f>
@@ -1432,58 +1447,58 @@
         <v>23</v>
       </c>
       <c r="E13" s="8" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="F13" s="9" t="s">
-        <v>158</v>
+        <v>156</v>
       </c>
       <c r="G13" s="8" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="H13" s="7" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="I13" s="10" t="s">
-        <v>159</v>
+        <v>157</v>
       </c>
       <c r="J13" s="7">
         <v>1</v>
       </c>
       <c r="K13" s="7"/>
     </row>
-    <row r="14" spans="1:11" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:11" ht="24.6" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A14" s="1"/>
       <c r="B14" s="11">
         <f t="shared" si="0"/>
         <v>12</v>
       </c>
       <c r="C14" s="13" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
       <c r="D14" s="9" t="s">
         <v>24</v>
       </c>
       <c r="E14" s="10" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="F14" s="9" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="G14" s="8" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="H14" s="9" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="I14" s="10" t="s">
-        <v>159</v>
+        <v>157</v>
       </c>
       <c r="J14" s="9">
         <v>6</v>
       </c>
       <c r="K14" s="9"/>
     </row>
-    <row r="15" spans="1:11" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:11" ht="24.6" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A15" s="1"/>
       <c r="B15" s="11">
         <f>ROW(B15) - ROW($B$2)</f>
@@ -1496,26 +1511,26 @@
         <v>25</v>
       </c>
       <c r="E15" s="8" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="F15" s="7" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="G15" s="8" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="H15" s="7" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="I15" s="10" t="s">
-        <v>159</v>
+        <v>157</v>
       </c>
       <c r="J15" s="7">
         <v>1</v>
       </c>
       <c r="K15" s="7"/>
     </row>
-    <row r="16" spans="1:11" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:11" ht="24.6" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A16" s="1"/>
       <c r="B16" s="11">
         <f t="shared" si="0"/>
@@ -1528,26 +1543,26 @@
         <v>26</v>
       </c>
       <c r="E16" s="10" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="F16" s="9" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="G16" s="10" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="H16" s="9" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="I16" s="10" t="s">
-        <v>159</v>
+        <v>157</v>
       </c>
       <c r="J16" s="9">
         <v>1</v>
       </c>
       <c r="K16" s="9"/>
     </row>
-    <row r="17" spans="1:11" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:11" ht="24.6" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A17" s="1"/>
       <c r="B17" s="11">
         <f>ROW(B17) - ROW($B$2)</f>
@@ -1560,26 +1575,26 @@
         <v>27</v>
       </c>
       <c r="E17" s="8" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="F17" s="7" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="G17" s="8" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="H17" s="7" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="I17" s="10" t="s">
-        <v>159</v>
+        <v>157</v>
       </c>
       <c r="J17" s="7">
         <v>1</v>
       </c>
       <c r="K17" s="7"/>
     </row>
-    <row r="18" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A18" s="1"/>
       <c r="B18" s="11">
         <f t="shared" si="0"/>
@@ -1588,32 +1603,32 @@
       <c r="C18" s="13" t="s">
         <v>8</v>
       </c>
-      <c r="D18" s="17" t="s">
+      <c r="D18" s="16" t="s">
         <v>28</v>
       </c>
-      <c r="E18" s="18" t="s">
-        <v>61</v>
-      </c>
-      <c r="F18" s="15" t="s">
+      <c r="E18" s="17" t="s">
+        <v>60</v>
+      </c>
+      <c r="F18" s="14" t="s">
+        <v>156</v>
+      </c>
+      <c r="G18" s="16" t="s">
+        <v>87</v>
+      </c>
+      <c r="H18" s="16" t="s">
+        <v>157</v>
+      </c>
+      <c r="I18" s="17" t="s">
+        <v>157</v>
+      </c>
+      <c r="J18" s="16">
+        <v>2</v>
+      </c>
+      <c r="K18" s="15" t="s">
         <v>158</v>
       </c>
-      <c r="G18" s="17" t="s">
-        <v>89</v>
-      </c>
-      <c r="H18" s="17" t="s">
-        <v>159</v>
-      </c>
-      <c r="I18" s="18" t="s">
-        <v>159</v>
-      </c>
-      <c r="J18" s="17">
-        <v>2</v>
-      </c>
-      <c r="K18" s="16" t="s">
-        <v>160</v>
-      </c>
-    </row>
-    <row r="19" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="19" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A19" s="1"/>
       <c r="B19" s="11">
         <f>ROW(B19) - ROW($B$2)</f>
@@ -1626,26 +1641,26 @@
         <v>29</v>
       </c>
       <c r="E19" s="8" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="F19" s="7" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="G19" s="8" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="H19" s="7" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
       <c r="I19" s="8" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="J19" s="7">
         <v>9</v>
       </c>
       <c r="K19" s="7"/>
     </row>
-    <row r="20" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A20" s="1"/>
       <c r="B20" s="11">
         <f t="shared" si="0"/>
@@ -1658,26 +1673,26 @@
         <v>30</v>
       </c>
       <c r="E20" s="10" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="F20" s="9" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="G20" s="10" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="H20" s="9" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
       <c r="I20" s="10" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="J20" s="9">
         <v>2</v>
       </c>
       <c r="K20" s="9"/>
     </row>
-    <row r="21" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A21" s="1"/>
       <c r="B21" s="11">
         <f>ROW(B21) - ROW($B$2)</f>
@@ -1690,26 +1705,26 @@
         <v>31</v>
       </c>
       <c r="E21" s="8" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="F21" s="7" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="G21" s="8" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="H21" s="7" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
       <c r="I21" s="8" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
       <c r="J21" s="7">
         <v>1</v>
       </c>
       <c r="K21" s="7"/>
     </row>
-    <row r="22" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A22" s="1"/>
       <c r="B22" s="11">
         <f t="shared" si="0"/>
@@ -1722,26 +1737,26 @@
         <v>32</v>
       </c>
       <c r="E22" s="10" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="F22" s="9" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="G22" s="10" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="H22" s="9" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
       <c r="I22" s="10" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="J22" s="9">
         <v>3</v>
       </c>
       <c r="K22" s="9"/>
     </row>
-    <row r="23" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A23" s="1"/>
       <c r="B23" s="11">
         <f>ROW(B23) - ROW($B$2)</f>
@@ -1754,26 +1769,26 @@
         <v>33</v>
       </c>
       <c r="E23" s="8" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="F23" s="7" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="G23" s="8" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="H23" s="7" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
       <c r="I23" s="8" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="J23" s="7">
         <v>2</v>
       </c>
       <c r="K23" s="7"/>
     </row>
-    <row r="24" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A24" s="1"/>
       <c r="B24" s="11">
         <f t="shared" si="0"/>
@@ -1786,26 +1801,26 @@
         <v>34</v>
       </c>
       <c r="E24" s="10" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="F24" s="9" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="G24" s="10" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="H24" s="9" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
       <c r="I24" s="10" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
       <c r="J24" s="9">
         <v>1</v>
       </c>
       <c r="K24" s="9"/>
     </row>
-    <row r="25" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A25" s="1"/>
       <c r="B25" s="11">
         <f>ROW(B25) - ROW($B$2)</f>
@@ -1818,26 +1833,26 @@
         <v>35</v>
       </c>
       <c r="E25" s="8" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="F25" s="7" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="G25" s="8" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="H25" s="7" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
       <c r="I25" s="8" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="J25" s="7">
         <v>1</v>
       </c>
       <c r="K25" s="7"/>
     </row>
-    <row r="26" spans="1:11" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:11" ht="24.6" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A26" s="1"/>
       <c r="B26" s="11">
         <f t="shared" si="0"/>
@@ -1850,26 +1865,26 @@
         <v>36</v>
       </c>
       <c r="E26" s="10" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="F26" s="9" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="G26" s="10" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="H26" s="9" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
       <c r="I26" s="10" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="J26" s="9">
         <v>2</v>
       </c>
       <c r="K26" s="9"/>
     </row>
-    <row r="27" spans="1:11" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:11" ht="24.6" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A27" s="1"/>
       <c r="B27" s="11">
         <f>ROW(B27) - ROW($B$2)</f>
@@ -1882,26 +1897,26 @@
         <v>37</v>
       </c>
       <c r="E27" s="8" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="F27" s="7" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="G27" s="8" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="H27" s="7" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
       <c r="I27" s="8" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="J27" s="7">
         <v>1</v>
       </c>
       <c r="K27" s="7"/>
     </row>
-    <row r="28" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A28" s="1"/>
       <c r="B28" s="11">
         <f t="shared" si="0"/>
@@ -1914,26 +1929,26 @@
         <v>38</v>
       </c>
       <c r="E28" s="10" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="F28" s="9" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="G28" s="10" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="H28" s="9" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
       <c r="I28" s="10" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
       <c r="J28" s="9">
         <v>1</v>
       </c>
       <c r="K28" s="9"/>
     </row>
-    <row r="29" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A29" s="1"/>
       <c r="B29" s="11">
         <f>ROW(B29) - ROW($B$2)</f>
@@ -1946,122 +1961,122 @@
         <v>39</v>
       </c>
       <c r="E29" s="8" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="F29" s="9" t="s">
-        <v>158</v>
+        <v>156</v>
       </c>
       <c r="G29" s="8" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="H29" s="7" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="I29" s="8" t="s">
-        <v>159</v>
+        <v>157</v>
       </c>
       <c r="J29" s="7">
         <v>1</v>
       </c>
       <c r="K29" s="7"/>
     </row>
-    <row r="30" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A30" s="1"/>
       <c r="B30" s="11">
         <f t="shared" si="0"/>
         <v>28</v>
       </c>
       <c r="C30" s="13" t="s">
-        <v>165</v>
+        <v>163</v>
       </c>
       <c r="D30" s="9" t="s">
         <v>40</v>
       </c>
       <c r="E30" s="10" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="F30" s="9" t="s">
-        <v>158</v>
+        <v>156</v>
       </c>
       <c r="G30" s="10" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="H30" s="9" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="I30" s="8" t="s">
-        <v>159</v>
+        <v>157</v>
       </c>
       <c r="J30" s="9">
         <v>1</v>
       </c>
       <c r="K30" s="9"/>
     </row>
-    <row r="31" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A31" s="1"/>
       <c r="B31" s="11">
         <f>ROW(B31) - ROW($B$2)</f>
         <v>29</v>
       </c>
       <c r="C31" s="13" t="s">
-        <v>165</v>
+        <v>163</v>
       </c>
       <c r="D31" s="7" t="s">
         <v>41</v>
       </c>
       <c r="E31" s="8" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="F31" s="9" t="s">
-        <v>158</v>
+        <v>156</v>
       </c>
       <c r="G31" s="8" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="H31" s="7" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="I31" s="8" t="s">
-        <v>159</v>
+        <v>157</v>
       </c>
       <c r="J31" s="7">
         <v>1</v>
       </c>
       <c r="K31" s="7"/>
     </row>
-    <row r="32" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A32" s="1"/>
       <c r="B32" s="11">
         <f t="shared" si="0"/>
         <v>30</v>
       </c>
       <c r="C32" s="13" t="s">
-        <v>165</v>
+        <v>163</v>
       </c>
       <c r="D32" s="9" t="s">
         <v>42</v>
       </c>
       <c r="E32" s="10" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="F32" s="9" t="s">
-        <v>158</v>
+        <v>156</v>
       </c>
       <c r="G32" s="10" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="H32" s="9" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="I32" s="8" t="s">
-        <v>159</v>
+        <v>157</v>
       </c>
       <c r="J32" s="9">
         <v>1</v>
       </c>
       <c r="K32" s="9"/>
     </row>
-    <row r="33" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A33" s="1"/>
       <c r="B33" s="11">
         <f>ROW(B33) - ROW($B$2)</f>
@@ -2074,26 +2089,26 @@
         <v>43</v>
       </c>
       <c r="E33" s="8" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="F33" s="9" t="s">
-        <v>158</v>
+        <v>156</v>
       </c>
       <c r="G33" s="9" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="H33" s="9" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="I33" s="8" t="s">
-        <v>154</v>
+        <v>152</v>
       </c>
       <c r="J33" s="7">
         <v>1</v>
       </c>
       <c r="K33" s="7"/>
     </row>
-    <row r="34" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A34" s="1"/>
       <c r="B34" s="11">
         <f t="shared" si="0"/>
@@ -2106,19 +2121,19 @@
         <v>44</v>
       </c>
       <c r="E34" s="10" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="F34" s="9" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="G34" s="10" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="H34" s="9" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="I34" s="10" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
       <c r="J34" s="9">
         <v>1</v>

</xml_diff>